<commit_message>
Basic writing to pdf from transaction ID
</commit_message>
<xml_diff>
--- a/DDDTools/DDDTools/data/datatable.xlsx
+++ b/DDDTools/DDDTools/data/datatable.xlsx
@@ -3706,8 +3706,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="000\-00\-0000"/>
+    <numFmt numFmtId="165" formatCode="00000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -3786,7 +3787,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -3840,6 +3841,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4201,7 +4205,7 @@
       <c r="A1" s="31">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="39" t="s">
         <v>39</v>
       </c>
       <c r="C1" s="1">
@@ -4216,7 +4220,7 @@
       <c r="F1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="2">
+      <c r="G1" s="40">
         <v>20020</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -4229,10 +4233,10 @@
         <v>43</v>
       </c>
       <c r="K1" s="1"/>
-      <c r="L1" s="29">
+      <c r="L1" s="41">
         <v>500</v>
       </c>
-      <c r="M1" s="35">
+      <c r="M1" s="29">
         <v>40686</v>
       </c>
       <c r="N1" s="1"/>

</xml_diff>

<commit_message>
+ dynamic number of rows + correct excel dates + correct amount of money format
</commit_message>
<xml_diff>
--- a/DDDTools/DDDTools/data/datatable.xlsx
+++ b/DDDTools/DDDTools/data/datatable.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="16925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Loren\Source\Repos\DDDTools\DDDTools\DDDTools\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lorenzo\Documents\DDDTools\DDDTools\DDDTools\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3887" uniqueCount="1216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3908" uniqueCount="1216">
   <si>
     <t>Epifani</t>
   </si>
@@ -26129,25 +26129,121 @@
       <c r="N584" s="1"/>
     </row>
     <row r="585" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A585"/>
-      <c r="B585"/>
-      <c r="G585"/>
-      <c r="L585"/>
-      <c r="M585"/>
+      <c r="A585" s="31">
+        <v>585</v>
+      </c>
+      <c r="B585" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C585" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D585" t="s">
+        <v>1213</v>
+      </c>
+      <c r="F585" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G585" s="2">
+        <v>20090</v>
+      </c>
+      <c r="H585" t="s">
+        <v>1212</v>
+      </c>
+      <c r="I585" t="s">
+        <v>42</v>
+      </c>
+      <c r="J585" s="28" t="s">
+        <v>1215</v>
+      </c>
+      <c r="K585" s="6" t="s">
+        <v>1215</v>
+      </c>
+      <c r="L585" s="29">
+        <v>500.1</v>
+      </c>
+      <c r="M585" s="35">
+        <v>42543</v>
+      </c>
+      <c r="N585" s="1"/>
     </row>
     <row r="586" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A586"/>
-      <c r="B586"/>
-      <c r="G586"/>
-      <c r="L586"/>
-      <c r="M586"/>
+      <c r="A586" s="31">
+        <v>586</v>
+      </c>
+      <c r="B586" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C586" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D586" t="s">
+        <v>1213</v>
+      </c>
+      <c r="F586" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G586" s="2">
+        <v>20090</v>
+      </c>
+      <c r="H586" t="s">
+        <v>1212</v>
+      </c>
+      <c r="I586" t="s">
+        <v>42</v>
+      </c>
+      <c r="J586" s="28" t="s">
+        <v>1215</v>
+      </c>
+      <c r="K586" s="6" t="s">
+        <v>1215</v>
+      </c>
+      <c r="L586" s="29">
+        <v>500.02</v>
+      </c>
+      <c r="M586" s="35">
+        <v>42543</v>
+      </c>
+      <c r="N586" s="1"/>
     </row>
     <row r="587" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A587"/>
-      <c r="B587"/>
-      <c r="G587"/>
-      <c r="L587"/>
-      <c r="M587"/>
+      <c r="A587" s="31">
+        <v>587</v>
+      </c>
+      <c r="B587" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C587" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D587" t="s">
+        <v>1213</v>
+      </c>
+      <c r="F587" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G587" s="2">
+        <v>20090</v>
+      </c>
+      <c r="H587" t="s">
+        <v>1212</v>
+      </c>
+      <c r="I587" t="s">
+        <v>42</v>
+      </c>
+      <c r="J587" s="28" t="s">
+        <v>1215</v>
+      </c>
+      <c r="K587" s="6" t="s">
+        <v>1215</v>
+      </c>
+      <c r="L587" s="29">
+        <v>500.78</v>
+      </c>
+      <c r="M587" s="35">
+        <v>42543</v>
+      </c>
+      <c r="N587" s="1"/>
     </row>
     <row r="588" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A588"/>
@@ -26183,6 +26279,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="landscape"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>